<commit_message>
Show Vyg Bound on port tiles and Summary sheet
- portTile now renders a "Vyg Bound <n>" line for the BKK/LCH ETA
  (and the alongside "NOW" case), fed from both the Python builder
  and the in-browser rebuild path.
- Summary sheet gains Vyg Bound columns for current call / THBKK / THLCH.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule - 9-9-SKED.xlsx
+++ b/Vessel Schedule - 9-9-SKED.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -447,11 +447,14 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,27 +485,42 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Vyg Bound</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ETA THBKK</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Wharf THBKK</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Vyg Bound THBKK</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ETA THLCH</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Wharf THLCH</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Vyg Bound THLCH</t>
         </is>
       </c>
     </row>
@@ -532,25 +550,38 @@
           <t>TWKEL -&gt; KRPUS</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-11T14:00:00</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>46287.91666666666</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2614N</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n">
         <v>46287.45833333334</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2614S</t>
         </is>
       </c>
     </row>
@@ -582,23 +613,38 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>0151S</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to VNSGN ~2026-09-10T05:00:00</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>46283.04166666666</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>0151N</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="n">
         <v>46282.52083333334</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>0151S</t>
         </is>
       </c>
     </row>
@@ -630,19 +676,32 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>2611S</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to IDJKT ~2026-09-11T22:00:00</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="2" t="n">
         <v/>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="J4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>46289.95833333334</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
         </is>
       </c>
     </row>
@@ -672,25 +731,38 @@
           <t>KRKAN -&gt; KRPUS</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-10-02T18:00:00</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="H5" s="3" t="n">
         <v>46308.375</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n">
         <v>46307.79166666666</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2612S</t>
         </is>
       </c>
     </row>
@@ -722,19 +794,32 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>2607S</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to VNSGN ~2026-09-11T20:00:00</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="2" t="n">
         <v/>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="J6" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K6" s="3" t="n">
         <v>46283.66666666666</v>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2607S</t>
         </is>
       </c>
     </row>
@@ -766,23 +851,38 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>2610S</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to THBKK ~2026-09-09T16:00:00</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="H7" s="3" t="n">
         <v>46274.75</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="n">
         <v>46276.79166666666</v>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
         </is>
       </c>
     </row>
@@ -812,25 +912,38 @@
           <t>CNXMN -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-11T07:00:00</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="H8" s="3" t="n">
         <v>46286.5625</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n">
         <v>46286.10416666666</v>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
         </is>
       </c>
     </row>
@@ -862,23 +975,38 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>2610S</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to HKHKG ~2026-09-10T18:00:00</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="H9" s="3" t="n">
         <v>46284.54166666666</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="n">
         <v>46284.08333333334</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
         </is>
       </c>
     </row>
@@ -908,21 +1036,32 @@
           <t>CNSHK -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-11T02:30:00</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="2" t="n">
         <v/>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="J10" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K10" s="3" t="n">
         <v>46294.75</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>2607S</t>
         </is>
       </c>
     </row>
@@ -952,25 +1091,38 @@
           <t>KRPUS -&gt; KRKAN</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-09T13:00:00</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="H11" s="3" t="n">
         <v>46283.70833333334</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n">
         <v>46283.33333333334</v>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2611S</t>
         </is>
       </c>
     </row>
@@ -1000,25 +1152,38 @@
           <t>VNSGN -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T12:00:00</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="H12" s="3" t="n">
         <v>46286</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2615N</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n">
         <v>46285.41666666666</v>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>2615S</t>
         </is>
       </c>
     </row>
@@ -1050,19 +1215,32 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>2607N</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to VNSGN ~2026-09-09T15:00:00</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="2" t="n">
         <v/>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="J13" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K13" s="3" t="n">
         <v>46304.70833333334</v>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
         </is>
       </c>
     </row>
@@ -1092,19 +1270,28 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>No data in window</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="2" t="n">
         <v/>
       </c>
-      <c r="I14" s="3" t="n"/>
       <c r="J14" s="2" t="n">
         <v/>
       </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="2" t="n">
+        <v/>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1132,25 +1319,38 @@
           <t>VNSGN -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-14T06:00:00</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="H15" s="3" t="n">
         <v>46281.67152777778</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n">
         <v>46281.66944444444</v>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>2609S</t>
         </is>
       </c>
     </row>
@@ -1182,23 +1382,38 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>2611S</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRKAN ~2026-09-09T21:00:00</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="H16" s="3" t="n">
         <v>46285.20833333334</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="n">
         <v>46284.6875</v>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>2611S</t>
         </is>
       </c>
     </row>
@@ -1230,23 +1445,38 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>2607N</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRPUS ~2026-09-10T10:00:00</t>
         </is>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="H17" s="3" t="n">
         <v>46292.5</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I17" s="3" t="n">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2608N</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n">
         <v>46291.91666666666</v>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>2608S</t>
         </is>
       </c>
     </row>
@@ -1278,23 +1508,38 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to THLCH ~2026-09-09T14:00:00</t>
         </is>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="H18" s="3" t="n">
         <v>46293.75</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I18" s="3" t="n">
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="n">
         <v>46274.79166666666</v>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
         </is>
       </c>
     </row>
@@ -1324,25 +1569,38 @@
           <t>KRPTK -&gt; KRKAN</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T02:00:00</t>
         </is>
       </c>
-      <c r="G19" s="3" t="n">
+      <c r="H19" s="3" t="n">
         <v>46284.41666666666</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I19" s="3" t="n">
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2615N</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="n">
         <v>46283.89583333334</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>2615S</t>
         </is>
       </c>
     </row>
@@ -1372,25 +1630,38 @@
           <t>VNSGN -&gt; THLCH</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T11:00:00</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n">
+      <c r="H20" s="3" t="n">
         <v>46275.91666666666</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="I20" s="3" t="n">
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="n">
         <v>46275.45833333334</v>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>LCH01</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>2609S</t>
         </is>
       </c>
     </row>
@@ -1420,25 +1691,38 @@
           <t>THLCH -&gt; HKHKG</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-13T01:00:00</t>
         </is>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="H21" s="3" t="n">
         <v>46293.125</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="I21" s="3" t="n">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="n">
         <v>46292.5</v>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
         </is>
       </c>
     </row>
@@ -1470,23 +1754,38 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
+          <t>2610S</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRKAN ~2026-09-09T16:00:00</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="H22" s="3" t="n">
         <v>46285.5</v>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I22" s="3" t="n">
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="n">
         <v>46285.125</v>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
         </is>
       </c>
     </row>
@@ -1518,23 +1817,38 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
+          <t>2609S</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to VNSGN ~2026-09-14T03:00:00</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="H23" s="3" t="n">
         <v>46287.16666666666</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="I23" s="3" t="n">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="n">
         <v>46286.54166666666</v>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>LCH01</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>2609S</t>
         </is>
       </c>
     </row>
@@ -1566,19 +1880,32 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
+          <t>2608N</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRPUS ~2026-09-12T18:30:00</t>
         </is>
       </c>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="2" t="n">
         <v/>
       </c>
-      <c r="I24" s="3" t="n">
+      <c r="J24" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K24" s="3" t="n">
         <v>46300.10416666666</v>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
         </is>
       </c>
     </row>
@@ -1610,23 +1937,38 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
+          <t>2608N</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRPTK ~2026-09-09T22:00:00</t>
         </is>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="H25" s="3" t="n">
         <v>46295.45833333334</v>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="I25" s="3" t="n">
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="n">
         <v>46294.83333333334</v>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>LCH01</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>2609S</t>
         </is>
       </c>
     </row>
@@ -1656,25 +1998,38 @@
           <t>KRKAN -&gt; HKHKG</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T04:00:00</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="H26" s="3" t="n">
         <v>46280.625</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I26" s="3" t="n">
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="n">
         <v>46280.16666666666</v>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>2610S</t>
         </is>
       </c>
     </row>
@@ -1704,21 +2059,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>No data in window</t>
         </is>
       </c>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="2" t="n">
         <v/>
       </c>
-      <c r="I27" s="3" t="n">
+      <c r="J27" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K27" s="3" t="n">
         <v>46297.375</v>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>2612N</t>
         </is>
       </c>
     </row>
@@ -1750,23 +2116,38 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to CNXMN ~2026-09-10T06:30:00</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="H28" s="3" t="n">
         <v>46289</v>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="I28" s="3" t="n">
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="n">
         <v>46288.625</v>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>2611S</t>
         </is>
       </c>
     </row>
@@ -1798,19 +2179,32 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
+          <t>2607S</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to VNSGN ~2026-09-15T03:00:00</t>
         </is>
       </c>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="2" t="n">
         <v/>
       </c>
-      <c r="I29" s="3" t="n">
+      <c r="J29" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K29" s="3" t="n">
         <v>46287</v>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>2607S</t>
         </is>
       </c>
     </row>
@@ -1842,17 +2236,28 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
+          <t>9002N</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRPUS ~2026-09-09T12:00:00</t>
         </is>
       </c>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="2" t="n">
         <v/>
       </c>
-      <c r="I30" s="3" t="n"/>
       <c r="J30" s="2" t="n">
         <v/>
       </c>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="2" t="n">
+        <v/>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1882,17 +2287,28 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
+          <t>2601N</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
           <t>Alongside, departs to KRPUS ~2026-09-11T04:00:00</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="3" t="n"/>
+      <c r="I31" s="2" t="n">
         <v/>
       </c>
-      <c r="I31" s="3" t="n"/>
       <c r="J31" s="2" t="n">
         <v/>
       </c>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="2" t="n">
+        <v/>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1920,19 +2336,28 @@
           <t>KRINC -&gt; CNTAO</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-15T09:00:00</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="2" t="n">
         <v/>
       </c>
-      <c r="I32" s="3" t="n"/>
       <c r="J32" s="2" t="n">
         <v/>
       </c>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="2" t="n">
+        <v/>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1960,21 +2385,32 @@
           <t>IDJKT -&gt; IDSRG</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="n">
+        <v/>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-09T15:00:00</t>
         </is>
       </c>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="2" t="n">
         <v/>
       </c>
-      <c r="I33" s="3" t="n">
+      <c r="J33" s="2" t="n">
+        <v/>
+      </c>
+      <c r="K33" s="3" t="n">
         <v>46279.54166666666</v>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>2607N</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add vessel short code (abbreviation)
The SKED "Vessel" column (e.g. KMBK for KMTC BANGKOK) now shows in
the card sub-line, the expanded panel title, and a new Summary-sheet
"Code" column, and is matched by the search box.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Vessel Schedule - 9-9-SKED.xlsx
+++ b/Vessel Schedule - 9-9-SKED.xlsx
@@ -439,22 +439,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,60 +466,65 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Op.Liner</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Current Location</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Vyg Bound</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ETA THBKK</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Wharf THBKK</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Vyg Bound THBKK</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ETA THLCH</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Wharf THLCH</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Vyg Bound THLCH</t>
         </is>
@@ -532,54 +538,59 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>CMA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>KTS1</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>TWKEL -&gt; KRPUS</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v/>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-11T14:00:00</t>
         </is>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>46287.91666666666</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>2614N</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>46287.45833333334</v>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>2614S</t>
         </is>
@@ -593,56 +604,61 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>NTX</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>DJS</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>KRPUS (PUS05)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>0151S</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to VNSGN ~2026-09-10T05:00:00</t>
         </is>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>46283.04166666666</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>0151N</t>
         </is>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>46282.52083333334</v>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>0151S</t>
         </is>
@@ -656,50 +672,55 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>HAB</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>HAS</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>CNSHA (SHAW1)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>2611S</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to IDJKT ~2026-09-11T22:00:00</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I4" s="3" t="n"/>
       <c r="J4" s="2" t="n">
         <v/>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="K4" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L4" s="3" t="n">
         <v>46289.95833333334</v>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
@@ -713,54 +734,59 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>HAHM</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>KHS1</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>HAS</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>KRKAN -&gt; KRPUS</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v/>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-10-02T18:00:00</t>
         </is>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="I5" s="3" t="n">
         <v>46308.375</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2612N</t>
         </is>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="L5" s="3" t="n">
         <v>46307.79166666666</v>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>2612S</t>
         </is>
@@ -774,50 +800,55 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>ICVY</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>ANX</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>CNSHA (SHAW5)</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>2607S</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to VNSGN ~2026-09-11T20:00:00</t>
         </is>
       </c>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I6" s="3" t="n"/>
       <c r="J6" s="2" t="n">
         <v/>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="K6" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L6" s="3" t="n">
         <v>46283.66666666666</v>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>2607S</t>
         </is>
@@ -831,56 +862,61 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>KTS1</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>THLCH (LCH04)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to THBKK ~2026-09-09T16:00:00</t>
         </is>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="I7" s="3" t="n">
         <v>46274.75</v>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="L7" s="3" t="n">
         <v>46276.79166666666</v>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
@@ -894,54 +930,59 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>KMGY</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>CHT</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>CNXMN -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v/>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-11T07:00:00</t>
         </is>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="I8" s="3" t="n">
         <v>46286.5625</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K8" s="3" t="n">
+      <c r="L8" s="3" t="n">
         <v>46286.10416666666</v>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
@@ -955,56 +996,61 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>KJT</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>KTS1</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>KRUSN (USN01)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to HKHKG ~2026-09-10T18:00:00</t>
         </is>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="I9" s="3" t="n">
         <v>46284.54166666666</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K9" s="3" t="n">
+      <c r="L9" s="3" t="n">
         <v>46284.08333333334</v>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
@@ -1018,48 +1064,53 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>KMSU</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>ANX</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>CNSHK -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v/>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-11T02:30:00</t>
         </is>
       </c>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I10" s="3" t="n"/>
       <c r="J10" s="2" t="n">
         <v/>
       </c>
-      <c r="K10" s="3" t="n">
+      <c r="K10" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L10" s="3" t="n">
         <v>46294.75</v>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>2607S</t>
         </is>
@@ -1073,54 +1124,59 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>KMTP</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>VTS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>KRPUS -&gt; KRKAN</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v/>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-09T13:00:00</t>
         </is>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="I11" s="3" t="n">
         <v>46283.70833333334</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="K11" s="3" t="n">
+      <c r="L11" s="3" t="n">
         <v>46283.33333333334</v>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>2611S</t>
         </is>
@@ -1134,54 +1190,59 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>KUS</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>KST</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>VNSGN -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v/>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T12:00:00</t>
         </is>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="I12" s="3" t="n">
         <v>46286</v>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2615N</t>
         </is>
       </c>
-      <c r="K12" s="3" t="n">
+      <c r="L12" s="3" t="n">
         <v>46285.41666666666</v>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>2615S</t>
         </is>
@@ -1195,50 +1256,55 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>KXM</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>ANX</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>KMT</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>IDJKT (JKT02)</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>2607N</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to VNSGN ~2026-09-09T15:00:00</t>
         </is>
       </c>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I13" s="3" t="n"/>
       <c r="J13" s="2" t="n">
         <v/>
       </c>
-      <c r="K13" s="3" t="n">
+      <c r="K13" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L13" s="3" t="n">
         <v>46304.70833333334</v>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>2608S</t>
         </is>
@@ -1252,46 +1318,51 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
+          <t>LCVY</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>nodata</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v/>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>No data in window</t>
         </is>
       </c>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I14" s="3" t="n"/>
       <c r="J14" s="2" t="n">
         <v/>
       </c>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="2" t="n">
+      <c r="K14" s="2" t="n">
         <v/>
       </c>
+      <c r="L14" s="3" t="n"/>
       <c r="M14" s="2" t="n">
         <v/>
       </c>
+      <c r="N14" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1301,54 +1372,59 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>PCCP</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>KST</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>PCS</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>VNSGN -&gt; KRINC</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v/>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-14T06:00:00</t>
         </is>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="I15" s="3" t="n">
         <v>46281.67152777778</v>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
       </c>
-      <c r="K15" s="3" t="n">
+      <c r="L15" s="3" t="n">
         <v>46281.66944444444</v>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>2609S</t>
         </is>
@@ -1362,56 +1438,61 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>PGPO</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>NTX</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>NAM</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>KRPTK (PTK02)</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>2611S</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRKAN ~2026-09-09T21:00:00</t>
         </is>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="I16" s="3" t="n">
         <v>46285.20833333334</v>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="K16" s="3" t="n">
+      <c r="L16" s="3" t="n">
         <v>46284.6875</v>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>2611S</t>
         </is>
@@ -1425,56 +1506,61 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>SWAL</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>KRPUS (PUS05)</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>2607N</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRPUS ~2026-09-10T10:00:00</t>
         </is>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="I17" s="3" t="n">
         <v>46292.5</v>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2608N</t>
         </is>
       </c>
-      <c r="K17" s="3" t="n">
+      <c r="L17" s="3" t="n">
         <v>46291.91666666666</v>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>2608S</t>
         </is>
@@ -1488,56 +1574,61 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
           <t>KTS1</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>THBKK (BKK01)</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to THLCH ~2026-09-09T14:00:00</t>
         </is>
       </c>
-      <c r="H18" s="3" t="n">
+      <c r="I18" s="3" t="n">
         <v>46293.75</v>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K18" s="3" t="n">
+      <c r="L18" s="3" t="n">
         <v>46274.79166666666</v>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
@@ -1551,54 +1642,59 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
+          <t>SWBT</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
           <t>NTX</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>KRPTK -&gt; KRKAN</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v/>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T02:00:00</t>
         </is>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="I19" s="3" t="n">
         <v>46284.41666666666</v>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2615N</t>
         </is>
       </c>
-      <c r="K19" s="3" t="n">
+      <c r="L19" s="3" t="n">
         <v>46283.89583333334</v>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>2615S</t>
         </is>
@@ -1612,54 +1708,59 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>SWCP</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
           <t>KST</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>VNSGN -&gt; THLCH</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v/>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T11:00:00</t>
         </is>
       </c>
-      <c r="H20" s="3" t="n">
+      <c r="I20" s="3" t="n">
         <v>46275.91666666666</v>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>BKK02</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
       </c>
-      <c r="K20" s="3" t="n">
+      <c r="L20" s="3" t="n">
         <v>46275.45833333334</v>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>LCH01</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>2609S</t>
         </is>
@@ -1673,54 +1774,59 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
+          <t>SWDN</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
           <t>CHT</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>THLCH -&gt; HKHKG</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v/>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-13T01:00:00</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="I21" s="3" t="n">
         <v>46293.125</v>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K21" s="3" t="n">
+      <c r="L21" s="3" t="n">
         <v>46292.5</v>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>LCH05</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
@@ -1734,56 +1840,61 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
+          <t>SWIC</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
           <t>KHS1</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>KRPUS (PUS05)</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRKAN ~2026-09-09T16:00:00</t>
         </is>
       </c>
-      <c r="H22" s="3" t="n">
+      <c r="I22" s="3" t="n">
         <v>46285.5</v>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K22" s="3" t="n">
+      <c r="L22" s="3" t="n">
         <v>46285.125</v>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
@@ -1797,56 +1908,61 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
           <t>BTS</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>CNSHA (SHAW1)</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>2609S</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to VNSGN ~2026-09-14T03:00:00</t>
         </is>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="I23" s="3" t="n">
         <v>46287.16666666666</v>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
       </c>
-      <c r="K23" s="3" t="n">
+      <c r="L23" s="3" t="n">
         <v>46286.54166666666</v>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>LCH01</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>2609S</t>
         </is>
@@ -1860,50 +1976,55 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
+          <t>SWRG</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>CNSHA (SHAW5)</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>2608N</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRPUS ~2026-09-12T18:30:00</t>
         </is>
       </c>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I24" s="3" t="n"/>
       <c r="J24" s="2" t="n">
         <v/>
       </c>
-      <c r="K24" s="3" t="n">
+      <c r="K24" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L24" s="3" t="n">
         <v>46300.10416666666</v>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
@@ -1917,56 +2038,61 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
+          <t>SWSP</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
           <t>BTS</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>VNSGN (SGN03)</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>2608N</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRPTK ~2026-09-09T22:00:00</t>
         </is>
       </c>
-      <c r="H25" s="3" t="n">
+      <c r="I25" s="3" t="n">
         <v>46295.45833333334</v>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>BKK04</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
       </c>
-      <c r="K25" s="3" t="n">
+      <c r="L25" s="3" t="n">
         <v>46294.83333333334</v>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>LCH01</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>2609S</t>
         </is>
@@ -1980,54 +2106,59 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
+          <t>SWSR</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
           <t>VTS</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>KRKAN -&gt; HKHKG</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v/>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-10T04:00:00</t>
         </is>
       </c>
-      <c r="H26" s="3" t="n">
+      <c r="I26" s="3" t="n">
         <v>46280.625</v>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="K26" s="3" t="n">
+      <c r="L26" s="3" t="n">
         <v>46280.16666666666</v>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>2610S</t>
         </is>
@@ -2041,48 +2172,53 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>SWVG</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>nodata</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="G27" s="2" t="n">
         <v/>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>No data in window</t>
         </is>
       </c>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I27" s="3" t="n"/>
       <c r="J27" s="2" t="n">
         <v/>
       </c>
-      <c r="K27" s="3" t="n">
+      <c r="K27" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L27" s="3" t="n">
         <v>46297.375</v>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>2612N</t>
         </is>
@@ -2096,56 +2232,61 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
+          <t>SKOR</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
           <t>VTS</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>CKL</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>HKHKG (HKG03)</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to CNXMN ~2026-09-10T06:30:00</t>
         </is>
       </c>
-      <c r="H28" s="3" t="n">
+      <c r="I28" s="3" t="n">
         <v>46289</v>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>BKK01</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="K28" s="3" t="n">
+      <c r="L28" s="3" t="n">
         <v>46288.625</v>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>2611S</t>
         </is>
@@ -2159,50 +2300,55 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>NSSJ</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
           <t>ANX</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>NAM</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>CNSHA (SHAW5)</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>2607S</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to VNSGN ~2026-09-15T03:00:00</t>
         </is>
       </c>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I29" s="3" t="n"/>
       <c r="J29" s="2" t="n">
         <v/>
       </c>
-      <c r="K29" s="3" t="n">
+      <c r="K29" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L29" s="3" t="n">
         <v>46287</v>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>LCH04</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>2607S</t>
         </is>
@@ -2216,48 +2362,53 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>SDBG</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>KRPUS (PUS05)</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>9002N</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRPUS ~2026-09-09T12:00:00</t>
         </is>
       </c>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I30" s="3" t="n"/>
       <c r="J30" s="2" t="n">
         <v/>
       </c>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="2" t="n">
+      <c r="K30" s="2" t="n">
         <v/>
       </c>
+      <c r="L30" s="3" t="n"/>
       <c r="M30" s="2" t="n">
         <v/>
       </c>
+      <c r="N30" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2267,48 +2418,53 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
+          <t>TJBG</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>HAS</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>docked</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>CNSHA (SHAW1)</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>2601N</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Alongside, departs to KRPUS ~2026-09-11T04:00:00</t>
         </is>
       </c>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I31" s="3" t="n"/>
       <c r="J31" s="2" t="n">
         <v/>
       </c>
-      <c r="K31" s="3" t="n"/>
-      <c r="L31" s="2" t="n">
+      <c r="K31" s="2" t="n">
         <v/>
       </c>
+      <c r="L31" s="3" t="n"/>
       <c r="M31" s="2" t="n">
         <v/>
       </c>
+      <c r="N31" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2318,46 +2474,51 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
+          <t>TSNA</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
           <t>CHT</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>TSL</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>KRINC -&gt; CNTAO</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v/>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-15T09:00:00</t>
         </is>
       </c>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I32" s="3" t="n"/>
       <c r="J32" s="2" t="n">
         <v/>
       </c>
-      <c r="K32" s="3" t="n"/>
-      <c r="L32" s="2" t="n">
+      <c r="K32" s="2" t="n">
         <v/>
       </c>
+      <c r="L32" s="3" t="n"/>
       <c r="M32" s="2" t="n">
         <v/>
       </c>
+      <c r="N32" s="2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2367,48 +2528,53 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t>YSVY</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
           <t>PCI2</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>SKR</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>transit</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>IDJKT -&gt; IDSRG</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v/>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>In transit, ETA 2026-09-09T15:00:00</t>
         </is>
       </c>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="2" t="n">
-        <v/>
-      </c>
+      <c r="I33" s="3" t="n"/>
       <c r="J33" s="2" t="n">
         <v/>
       </c>
-      <c r="K33" s="3" t="n">
+      <c r="K33" s="2" t="n">
+        <v/>
+      </c>
+      <c r="L33" s="3" t="n">
         <v>46279.54166666666</v>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>LCH06</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>2607N</t>
         </is>

</xml_diff>